<commit_message>
Add ACR and order values in AED/USD, country value chart, SLOB value
Order tracker gains an ACR (USD per case) column from Logistics.
Order, dispatch and balance values are calculated per order with
totals, shown in AED by default at an admin-set rate with a USD toggle.
Dashboard adds value tiles and a Country vs Value chart. The SLOB
sheet shows value from its own case rate or the tracker ACR.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnMbwzmej8r4PCq7VjYzE3
</commit_message>
<xml_diff>
--- a/docs/templates/fg-slob-template.xlsx
+++ b/docs/templates/fg-slob-template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -435,8 +435,9 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,10 +478,15 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Case Rate (USD)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>SLOB Category</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>

</xml_diff>